<commit_message>
Convert RPG example to Excel and CFD sources
</commit_message>
<xml_diff>
--- a/examples/rpg/data/rpg.xlsx
+++ b/examples/rpg/data/rpg.xlsx
@@ -2,16 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item" sheetId="1" r:id="R52dbdc023bce415c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="Rf531816d5cf84605"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buff" sheetId="3" r:id="R68e2e336839d48c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill" sheetId="4" r:id="R2d8088a070354357"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster" sheetId="5" r:id="R0be2e9de3b2f4d19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DropTable" sheetId="6" r:id="R3c95343529bf4055"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stage" sheetId="7" r:id="R56856c5aa9744163"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quest" sheetId="8" r:id="R2e2443ebd0524bb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shop" sheetId="9" r:id="R15bab0945dcd4a52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="10" r:id="Rdf3710ed718843a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item" sheetId="1" r:id="Rb7cbc0639c1244cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R7769ea97feba4da2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Buff" sheetId="3" r:id="R296ef19d76494114"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skill" sheetId="4" r:id="Rb566210011db4cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monster" sheetId="5" r:id="R9a0ba626eda14e38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="6" r:id="Rd6964cd1ea5e4311"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -321,6 +317,9 @@
         <x:v>Upgrade Item ID</x:v>
       </x:c>
       <x:c r="M1" s="2" t="str">
+        <x:v>Featured Stage ID</x:v>
+      </x:c>
+      <x:c r="N1" s="2" t="str">
         <x:v>Legacy Power</x:v>
       </x:c>
     </x:row>
@@ -361,7 +360,10 @@
       <x:c r="L2" t="str">
         <x:v>_</x:v>
       </x:c>
-      <x:c r="M2" t="n">
+      <x:c r="M2" t="str">
+        <x:v>@Stage.stage_forest_road</x:v>
+      </x:c>
+      <x:c r="N2" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -402,7 +404,10 @@
       <x:c r="L3" t="str">
         <x:v>_</x:v>
       </x:c>
-      <x:c r="M3" t="n">
+      <x:c r="M3" t="str">
+        <x:v>@Stage.stage_arcane_tower</x:v>
+      </x:c>
+      <x:c r="N3" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -443,357 +448,11 @@
       <x:c r="L4" t="str">
         <x:v>_</x:v>
       </x:c>
-      <x:c r="M4" t="n">
+      <x:c r="M4" t="str">
+        <x:v>@Stage.stage_dragon_peak</x:v>
+      </x:c>
+      <x:c r="N4" t="n">
         <x:v>120</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2" t="str">
-        <x:v>Text ID</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="str">
-        <x:v>ZH-CN</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>EN-US</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>Context</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
-        <x:v>Max Length</x:v>
-      </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>Tags</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>item_iron_sword_name</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>铁剑</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>Iron Sword</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
-        <x:v>equipment name</x:v>
-      </x:c>
-      <x:c r="E2" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F2" t="str">
-        <x:v>item | equipment</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>item_flame_staff_name</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>焰火法杖</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>Flame Staff</x:v>
-      </x:c>
-      <x:c r="D3" t="str">
-        <x:v>equipment name</x:v>
-      </x:c>
-      <x:c r="E3" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F3" t="str">
-        <x:v>item | equipment</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>item_meteor_staff_name</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>陨星法杖</x:v>
-      </x:c>
-      <x:c r="C4" t="str">
-        <x:v>Meteor Staff</x:v>
-      </x:c>
-      <x:c r="D4" t="str">
-        <x:v>equipment name</x:v>
-      </x:c>
-      <x:c r="E4" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F4" t="str">
-        <x:v>item | equipment</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>item_dragon_guard_name</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>龙鳞护甲</x:v>
-      </x:c>
-      <x:c r="C5" t="str">
-        <x:v>Dragon Guard</x:v>
-      </x:c>
-      <x:c r="D5" t="str">
-        <x:v>equipment name</x:v>
-      </x:c>
-      <x:c r="E5" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F5" t="str">
-        <x:v>item | equipment</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>buff_burning_name</x:v>
-      </x:c>
-      <x:c r="B6" t="str">
-        <x:v>燃烧</x:v>
-      </x:c>
-      <x:c r="C6" t="str">
-        <x:v>Burning</x:v>
-      </x:c>
-      <x:c r="D6" t="str">
-        <x:v>buff name</x:v>
-      </x:c>
-      <x:c r="E6" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F6" t="str">
-        <x:v>buff | combat</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>buff_battle_focus_name</x:v>
-      </x:c>
-      <x:c r="B7" t="str">
-        <x:v>战斗专注</x:v>
-      </x:c>
-      <x:c r="C7" t="str">
-        <x:v>Battle Focus</x:v>
-      </x:c>
-      <x:c r="D7" t="str">
-        <x:v>buff name</x:v>
-      </x:c>
-      <x:c r="E7" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F7" t="str">
-        <x:v>buff | combat</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>buff_meteor_mark_name</x:v>
-      </x:c>
-      <x:c r="B8" t="str">
-        <x:v>陨星印记</x:v>
-      </x:c>
-      <x:c r="C8" t="str">
-        <x:v>Meteor Mark</x:v>
-      </x:c>
-      <x:c r="D8" t="str">
-        <x:v>buff name</x:v>
-      </x:c>
-      <x:c r="E8" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F8" t="str">
-        <x:v>buff | raid</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>stage_forest_road_name</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>林地道路</x:v>
-      </x:c>
-      <x:c r="C9" t="str">
-        <x:v>Forest Road</x:v>
-      </x:c>
-      <x:c r="D9" t="str">
-        <x:v>stage name</x:v>
-      </x:c>
-      <x:c r="E9" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F9" t="str">
-        <x:v>stage | story</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>stage_arcane_tower_name</x:v>
-      </x:c>
-      <x:c r="B10" t="str">
-        <x:v>秘法高塔</x:v>
-      </x:c>
-      <x:c r="C10" t="str">
-        <x:v>Arcane Tower</x:v>
-      </x:c>
-      <x:c r="D10" t="str">
-        <x:v>stage name</x:v>
-      </x:c>
-      <x:c r="E10" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F10" t="str">
-        <x:v>stage | elite</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>stage_dragon_peak_name</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>龙巢峰顶</x:v>
-      </x:c>
-      <x:c r="C11" t="str">
-        <x:v>Dragon Peak</x:v>
-      </x:c>
-      <x:c r="D11" t="str">
-        <x:v>stage name</x:v>
-      </x:c>
-      <x:c r="E11" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F11" t="str">
-        <x:v>stage | raid</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>quest_first_blade_title</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:v>第一把剑</x:v>
-      </x:c>
-      <x:c r="C12" t="str">
-        <x:v>First Blade</x:v>
-      </x:c>
-      <x:c r="D12" t="str">
-        <x:v>quest title</x:v>
-      </x:c>
-      <x:c r="E12" t="n">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="F12" t="str">
-        <x:v>quest | story</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>quest_mage_trial_title</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>法师试炼</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
-        <x:v>Mage Trial</x:v>
-      </x:c>
-      <x:c r="D13" t="str">
-        <x:v>quest title</x:v>
-      </x:c>
-      <x:c r="E13" t="n">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="F13" t="str">
-        <x:v>quest | side</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>quest_dragon_raid_title</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>巨龙讨伐</x:v>
-      </x:c>
-      <x:c r="C14" t="str">
-        <x:v>Dragon Raid</x:v>
-      </x:c>
-      <x:c r="D14" t="str">
-        <x:v>quest title</x:v>
-      </x:c>
-      <x:c r="E14" t="n">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="F14" t="str">
-        <x:v>quest | raid</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>shop_starter_name</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>新手补给</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
-        <x:v>Starter Supply</x:v>
-      </x:c>
-      <x:c r="D15" t="str">
-        <x:v>shop name</x:v>
-      </x:c>
-      <x:c r="E15" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F15" t="str">
-        <x:v>shop | general</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>shop_arcane_name</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>秘法商店</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>Arcane Shop</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>shop name</x:v>
-      </x:c>
-      <x:c r="E16" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F16" t="str">
-        <x:v>shop | event</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>shop_raid_name</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>讨伐补给</x:v>
-      </x:c>
-      <x:c r="C17" t="str">
-        <x:v>Raid Supply</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
-        <x:v>shop name</x:v>
-      </x:c>
-      <x:c r="E17" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="F17" t="str">
-        <x:v>shop | raid</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -846,21 +505,24 @@
         <x:v>Upgrade Item ID</x:v>
       </x:c>
       <x:c r="N1" s="2" t="str">
+        <x:v>Featured Stage ID</x:v>
+      </x:c>
+      <x:c r="O1" s="2" t="str">
         <x:v>Legacy Power</x:v>
       </x:c>
-      <x:c r="O1" s="2" t="str">
+      <x:c r="P1" s="2" t="str">
         <x:v>Required Class</x:v>
       </x:c>
-      <x:c r="P1" s="2" t="str">
+      <x:c r="Q1" s="2" t="str">
         <x:v>Stat Bonus</x:v>
       </x:c>
-      <x:c r="Q1" s="2" t="str">
+      <x:c r="R1" s="2" t="str">
         <x:v>Allowed Classes</x:v>
       </x:c>
-      <x:c r="R1" s="2" t="str">
+      <x:c r="S1" s="2" t="str">
         <x:v>Upgrade Costs</x:v>
       </x:c>
-      <x:c r="S1" s="2" t="str">
+      <x:c r="T1" s="2" t="str">
         <x:v>Set Piece ID</x:v>
       </x:c>
     </x:row>
@@ -904,22 +566,25 @@
       <x:c r="M2" t="str">
         <x:v>@Equipment.flame_staff</x:v>
       </x:c>
-      <x:c r="N2" t="n">
+      <x:c r="N2" t="str">
+        <x:v>@Stage.stage_forest_road</x:v>
+      </x:c>
+      <x:c r="O2" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="O2" t="str">
+      <x:c r="P2" t="str">
         <x:v>warrior</x:v>
       </x:c>
-      <x:c r="P2" t="str">
+      <x:c r="Q2" t="str">
         <x:v>hp: 10, attack: 12, defense: 2, speed: 1.0, crit: 5</x:v>
       </x:c>
-      <x:c r="Q2" t="str">
+      <x:c r="R2" t="str">
         <x:v>warrior | ranger</x:v>
       </x:c>
-      <x:c r="R2" t="str">
+      <x:c r="S2" t="str">
         <x:v>1: 40, 2: 80, 3: 160</x:v>
       </x:c>
-      <x:c r="S2" t="str">
+      <x:c r="T2" t="str">
         <x:v>_</x:v>
       </x:c>
     </x:row>
@@ -963,22 +628,25 @@
       <x:c r="M3" t="str">
         <x:v>@Equipment.meteor_staff</x:v>
       </x:c>
-      <x:c r="N3" t="n">
+      <x:c r="N3" t="str">
+        <x:v>@Stage.stage_arcane_tower</x:v>
+      </x:c>
+      <x:c r="O3" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="O3" t="str">
+      <x:c r="P3" t="str">
         <x:v>mage</x:v>
       </x:c>
-      <x:c r="P3" t="str">
+      <x:c r="Q3" t="str">
         <x:v>hp: 12, attack: 48, defense: 4, speed: 0.9, crit: 8</x:v>
       </x:c>
-      <x:c r="Q3" t="str">
+      <x:c r="R3" t="str">
         <x:v>mage | scholar</x:v>
       </x:c>
-      <x:c r="R3" t="str">
+      <x:c r="S3" t="str">
         <x:v>1: 120, 2: 240, 3: 480</x:v>
       </x:c>
-      <x:c r="S3" t="str">
+      <x:c r="T3" t="str">
         <x:v>_</x:v>
       </x:c>
     </x:row>
@@ -1022,22 +690,25 @@
       <x:c r="M4" t="str">
         <x:v>_</x:v>
       </x:c>
-      <x:c r="N4" t="n">
+      <x:c r="N4" t="str">
+        <x:v>@Stage.stage_dragon_peak</x:v>
+      </x:c>
+      <x:c r="O4" t="n">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="O4" t="str">
+      <x:c r="P4" t="str">
         <x:v>mage</x:v>
       </x:c>
-      <x:c r="P4" t="str">
+      <x:c r="Q4" t="str">
         <x:v>hp: 40, attack: 96, defense: 18, speed: 0.8, crit: 18</x:v>
       </x:c>
-      <x:c r="Q4" t="str">
+      <x:c r="R4" t="str">
         <x:v>mage | scholar</x:v>
       </x:c>
-      <x:c r="R4" t="str">
+      <x:c r="S4" t="str">
         <x:v>1: 300, 2: 600, 3: 900</x:v>
       </x:c>
-      <x:c r="S4" t="str">
+      <x:c r="T4" t="str">
         <x:v>_</x:v>
       </x:c>
     </x:row>
@@ -1081,22 +752,25 @@
       <x:c r="M5" t="str">
         <x:v>_</x:v>
       </x:c>
-      <x:c r="N5" t="n">
+      <x:c r="N5" t="str">
+        <x:v>@Stage.stage_dragon_peak</x:v>
+      </x:c>
+      <x:c r="O5" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="O5" t="str">
+      <x:c r="P5" t="str">
         <x:v>warrior</x:v>
       </x:c>
-      <x:c r="P5" t="str">
+      <x:c r="Q5" t="str">
         <x:v>hp: 220, attack: 12, defense: 160, speed: 0.7, crit: 4</x:v>
       </x:c>
-      <x:c r="Q5" t="str">
+      <x:c r="R5" t="str">
         <x:v>warrior | guardian</x:v>
       </x:c>
-      <x:c r="R5" t="str">
+      <x:c r="S5" t="str">
         <x:v>1: 500, 2: 750, 3: 950</x:v>
       </x:c>
-      <x:c r="S5" t="str">
+      <x:c r="T5" t="str">
         <x:v>@Equipment.iron_sword</x:v>
       </x:c>
     </x:row>
@@ -1659,541 +1333,342 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Drop ID</x:v>
+        <x:v>Text ID</x:v>
       </x:c>
       <x:c r="B1" s="2" t="str">
-        <x:v>Monster ID</x:v>
+        <x:v>ZH-CN</x:v>
       </x:c>
       <x:c r="C1" s="2" t="str">
-        <x:v>Conditions</x:v>
+        <x:v>EN-US</x:v>
       </x:c>
       <x:c r="D1" s="2" t="str">
-        <x:v>Rewards</x:v>
+        <x:v>Context</x:v>
       </x:c>
       <x:c r="E1" s="2" t="str">
-        <x:v>Weights</x:v>
+        <x:v>Max Length</x:v>
       </x:c>
       <x:c r="F1" s="2" t="str">
-        <x:v>Bonus By Rarity</x:v>
-      </x:c>
-      <x:c r="G1" s="2" t="str">
-        <x:v>Currency Curve</x:v>
-      </x:c>
-      <x:c r="H1" s="2" t="str">
-        <x:v>Guaranteed Reward</x:v>
-      </x:c>
-      <x:c r="I1" s="2" t="str">
-        <x:v>Notes</x:v>
+        <x:v>Tags</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>drop_goblin_warrior</x:v>
+        <x:v>item_iron_sword_name</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>@Monster.goblin_warrior</x:v>
+        <x:v>铁剑</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>min_level: 1, required_element: Physical, flags: Damage</x:v>
+        <x:v>Iron Sword</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>ItemReward{key: reward_goblin_sword, item: @Equipment.iron_sword, count: 1} | CurrencyReward{key: reward_goblin_gold, count: 1, currency: gold, amount: 35}</x:v>
-      </x:c>
-      <x:c r="E2" t="str">
-        <x:v>70 | 30</x:v>
+        <x:v>equipment name</x:v>
+      </x:c>
+      <x:c r="E2" t="n">
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>Common: 0, Rare: 5</x:v>
-      </x:c>
-      <x:c r="G2" t="str">
-        <x:v>1: 10, 5: 20</x:v>
-      </x:c>
-      <x:c r="H2" t="str">
-        <x:v>CurrencyReward{key: guaranteed_goblin_gold, count: 1, currency: gold, amount: 5}</x:v>
-      </x:c>
-      <x:c r="I2" t="str">
-        <x:v>tutorial | melee</x:v>
+        <x:v>item | equipment</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>drop_fire_mage</x:v>
+        <x:v>item_flame_staff_name</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>@Monster.fire_mage</x:v>
+        <x:v>焰火法杖</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>min_level: 12, required_element: Fire, flags: Damage</x:v>
+        <x:v>Flame Staff</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>ItemReward{key: reward_mage_staff, item: @Equipment.flame_staff, count: 1} | CurrencyReward{key: reward_mage_gold, count: 1, currency: gold, amount: 120} | SkillUnlockReward{key: reward_mage_skill, skill: @Skill.fireball, required_level: 12}</x:v>
-      </x:c>
-      <x:c r="E3" t="str">
-        <x:v>25 | 65 | 10</x:v>
+        <x:v>equipment name</x:v>
+      </x:c>
+      <x:c r="E3" t="n">
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>Common: 0, Rare: 15, Epic: 30</x:v>
-      </x:c>
-      <x:c r="G3" t="str">
-        <x:v>1: 25, 18: 90</x:v>
-      </x:c>
-      <x:c r="H3" t="str">
-        <x:v>ItemReward{key: guaranteed_mage_staff, item: @Equipment.flame_staff, count: 1}</x:v>
-      </x:c>
-      <x:c r="I3" t="str">
-        <x:v>caster | fire</x:v>
+        <x:v>item | equipment</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>drop_ancient_dragon</x:v>
+        <x:v>item_meteor_staff_name</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>@Monster.ancient_dragon</x:v>
+        <x:v>陨星法杖</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>min_level: 45, required_element: Fire, flags: Ultimate</x:v>
+        <x:v>Meteor Staff</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>ItemReward{key: reward_dragon_feather, item: @Item.phoenix_feather, count: 2} | CurrencyReward{key: reward_dragon_gold, count: 1, currency: gold, amount: 1000} | SkillUnlockReward{key: reward_dragon_meteor, skill: @Skill.meteor, required_level: 45}</x:v>
-      </x:c>
-      <x:c r="E4" t="str">
-        <x:v>40 | 45 | 15</x:v>
+        <x:v>equipment name</x:v>
+      </x:c>
+      <x:c r="E4" t="n">
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>Common: 0, Rare: 30, Epic: 80, Legendary: 120</x:v>
-      </x:c>
-      <x:c r="G4" t="str">
-        <x:v>1: 100, 50: 900</x:v>
-      </x:c>
-      <x:c r="H4" t="str">
-        <x:v>ItemReward{key: guaranteed_dragon_scale, item: @Item.dragon_scale, count: 1}</x:v>
-      </x:c>
-      <x:c r="I4" t="str">
-        <x:v>raid | dragon | endgame</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2" t="str">
-        <x:v>Stage ID</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="str">
-        <x:v>Name Text ID</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>Kind</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>Unlock Level</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
-        <x:v>Recommended Power</x:v>
-      </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>Positions</x:v>
-      </x:c>
-      <x:c r="G1" s="2" t="str">
-        <x:v>Spawns</x:v>
-      </x:c>
-      <x:c r="H1" s="2" t="str">
-        <x:v>Drop Table ID</x:v>
-      </x:c>
-      <x:c r="I1" s="2" t="str">
-        <x:v>First Clear Reward</x:v>
-      </x:c>
-      <x:c r="J1" s="2" t="str">
-        <x:v>Modifiers</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>stage_forest_road</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>@Text.stage_forest_road_name</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="D2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" t="n">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="F2" t="str">
-        <x:v>{x: 9.0, y: 4.0}</x:v>
-      </x:c>
-      <x:c r="G2" t="str">
-        <x:v>{monster: @Monster.goblin_warrior, count: 3, level_offset: 0, weight: 100}</x:v>
-      </x:c>
-      <x:c r="H2" t="str">
-        <x:v>@DropTable.drop_goblin_warrior</x:v>
-      </x:c>
-      <x:c r="I2" t="str">
-        <x:v>ItemReward{key: first_clear_forest_blade, item: @Equipment.iron_sword, count: 1}</x:v>
-      </x:c>
-      <x:c r="J2" t="str">
-        <x:v>stamina: 6, time_limit: 300</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>stage_arcane_tower</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>@Text.stage_arcane_tower_name</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>Elite</x:v>
-      </x:c>
-      <x:c r="D3" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E3" t="n">
-        <x:v>260</x:v>
-      </x:c>
-      <x:c r="F3" t="str">
-        <x:v>{x: 20.0, y: -7.0} | {x: 25.0, y: -9.0}</x:v>
-      </x:c>
-      <x:c r="G3" t="str">
-        <x:v>{monster: @Monster.fire_mage, count: 1, level_offset: 0, weight: 70} | {monster: @Monster.goblin_warrior, count: 2, level_offset: 3, weight: 30}</x:v>
-      </x:c>
-      <x:c r="H3" t="str">
-        <x:v>@DropTable.drop_fire_mage</x:v>
-      </x:c>
-      <x:c r="I3" t="str">
-        <x:v>SkillUnlockReward{key: first_clear_fireball, skill: @Skill.fireball, required_level: 12}</x:v>
-      </x:c>
-      <x:c r="J3" t="str">
-        <x:v>stamina: 12, time_limit: 420</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>stage_dragon_peak</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>@Text.stage_dragon_peak_name</x:v>
-      </x:c>
-      <x:c r="C4" t="str">
-        <x:v>Raid</x:v>
-      </x:c>
-      <x:c r="D4" t="n">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E4" t="n">
-        <x:v>900</x:v>
-      </x:c>
-      <x:c r="F4" t="str">
-        <x:v>{x: 61.0, y: 79.0} | {x: 80.0, y: 90.0}</x:v>
-      </x:c>
-      <x:c r="G4" t="str">
-        <x:v>{monster: @Monster.ancient_dragon, count: 1, level_offset: 0, weight: 100} | {monster: @Monster.fire_mage, count: 2, level_offset: 5, weight: 20}</x:v>
-      </x:c>
-      <x:c r="H4" t="str">
-        <x:v>@DropTable.drop_ancient_dragon</x:v>
-      </x:c>
-      <x:c r="I4" t="str">
-        <x:v>ItemReward{key: first_clear_dragon_scale, item: @Item.dragon_scale, count: 1}</x:v>
-      </x:c>
-      <x:c r="J4" t="str">
-        <x:v>stamina: 30, time_limit: 900, raid_size: 4</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2" t="str">
-        <x:v>Quest ID</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="str">
-        <x:v>Kind</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>Title Text ID</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>Title</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
-        <x:v>Min Level</x:v>
-      </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>Stage ID</x:v>
-      </x:c>
-      <x:c r="G1" s="2" t="str">
-        <x:v>Target Monster ID</x:v>
-      </x:c>
-      <x:c r="H1" s="2" t="str">
-        <x:v>Reward Item ID</x:v>
-      </x:c>
-      <x:c r="I1" s="2" t="str">
-        <x:v>Prerequisites</x:v>
-      </x:c>
-      <x:c r="J1" s="2" t="str">
-        <x:v>Objectives</x:v>
-      </x:c>
-      <x:c r="K1" s="2" t="str">
-        <x:v>Reward Preview</x:v>
-      </x:c>
-      <x:c r="L1" s="2" t="str">
-        <x:v>Availability</x:v>
-      </x:c>
-      <x:c r="M1" s="2" t="str">
-        <x:v>Dialogue</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>quest_first_blade</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>Story</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>@Text.quest_first_blade_title</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
+        <x:v>item | equipment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>item_dragon_guard_name</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>龙鳞护甲</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Dragon Guard</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>equipment name</x:v>
+      </x:c>
+      <x:c r="E5" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>item | equipment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>buff_burning_name</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>燃烧</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Burning</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>buff name</x:v>
+      </x:c>
+      <x:c r="E6" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>buff | combat</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>buff_battle_focus_name</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>战斗专注</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Battle Focus</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>buff name</x:v>
+      </x:c>
+      <x:c r="E7" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>buff | combat</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>buff_meteor_mark_name</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>陨星印记</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Meteor Mark</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>buff name</x:v>
+      </x:c>
+      <x:c r="E8" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>buff | raid</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>stage_forest_road_name</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>林地道路</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Forest Road</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>stage name</x:v>
+      </x:c>
+      <x:c r="E9" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>stage | story</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>stage_arcane_tower_name</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>秘法高塔</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Arcane Tower</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>stage name</x:v>
+      </x:c>
+      <x:c r="E10" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>stage | elite</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>stage_dragon_peak_name</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>龙巢峰顶</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Dragon Peak</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>stage name</x:v>
+      </x:c>
+      <x:c r="E11" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>stage | raid</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>quest_first_blade_title</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>第一把剑</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
         <x:v>First Blade</x:v>
       </x:c>
-      <x:c r="E2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" t="str">
-        <x:v>@Stage.stage_forest_road</x:v>
-      </x:c>
-      <x:c r="G2" t="str">
-        <x:v>@Monster.goblin_warrior</x:v>
-      </x:c>
-      <x:c r="H2" t="str">
-        <x:v>@Equipment.iron_sword</x:v>
-      </x:c>
-      <x:c r="I2" t="str">
-        <x:v>_</x:v>
-      </x:c>
-      <x:c r="J2" t="str">
-        <x:v>{key: defeat_goblins, target_count: 3, counters: {kill: 3, collect: 0}}</x:v>
-      </x:c>
-      <x:c r="K2" t="str">
-        <x:v>ItemReward{key: preview_first_blade, item: @Equipment.iron_sword, count: 1}</x:v>
-      </x:c>
-      <x:c r="L2" t="str">
-        <x:v>start_day: 1, end_day: 30</x:v>
-      </x:c>
-      <x:c r="M2" t="str">
-        <x:v>key: root, text: "Clear the road.", next: [{key: accept, text: "I will handle it."} | {key: decline, text: "Later."}]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>quest_mage_trial</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>Side</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>@Text.quest_mage_trial_title</x:v>
-      </x:c>
-      <x:c r="D3" t="str">
+      <x:c r="D12" t="str">
+        <x:v>quest title</x:v>
+      </x:c>
+      <x:c r="E12" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>quest | story</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>quest_mage_trial_title</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>法师试炼</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
         <x:v>Mage Trial</x:v>
       </x:c>
-      <x:c r="E3" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="F3" t="str">
-        <x:v>@Stage.stage_arcane_tower</x:v>
-      </x:c>
-      <x:c r="G3" t="str">
-        <x:v>@Monster.fire_mage</x:v>
-      </x:c>
-      <x:c r="H3" t="str">
-        <x:v>@Equipment.flame_staff</x:v>
-      </x:c>
-      <x:c r="I3" t="str">
-        <x:v>quest_first_blade</x:v>
-      </x:c>
-      <x:c r="J3" t="str">
-        <x:v>{key: defeat_mage, target_count: 1, counters: {kill: 1}} | {key: collect_focus, target_count: 2, counters: {collect: 2, kill: 0}}</x:v>
-      </x:c>
-      <x:c r="K3" t="str">
-        <x:v>SkillUnlockReward{key: preview_mage_skill, skill: @Skill.fireball, required_level: 12}</x:v>
-      </x:c>
-      <x:c r="L3" t="str">
-        <x:v>start_day: 5, end_day: 45</x:v>
-      </x:c>
-      <x:c r="M3" t="str">
-        <x:v>key: root, text: "Prove your focus.", next: [{key: teach, text: "Show me the spell."}]</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>quest_dragon_raid</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>Raid</x:v>
-      </x:c>
-      <x:c r="C4" t="str">
-        <x:v>@Text.quest_dragon_raid_title</x:v>
-      </x:c>
-      <x:c r="D4" t="str">
+      <x:c r="D13" t="str">
+        <x:v>quest title</x:v>
+      </x:c>
+      <x:c r="E13" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>quest | side</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>quest_dragon_raid_title</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>巨龙讨伐</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
         <x:v>Dragon Raid</x:v>
       </x:c>
-      <x:c r="E4" t="n">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="F4" t="str">
-        <x:v>@Stage.stage_dragon_peak</x:v>
-      </x:c>
-      <x:c r="G4" t="str">
-        <x:v>@Monster.ancient_dragon</x:v>
-      </x:c>
-      <x:c r="H4" t="str">
-        <x:v>@Item.dragon_scale</x:v>
-      </x:c>
-      <x:c r="I4" t="str">
-        <x:v>quest_first_blade | quest_mage_trial</x:v>
-      </x:c>
-      <x:c r="J4" t="str">
-        <x:v>{key: break_wings, target_count: 2, counters: {kill: 1, collect: 2}} | {key: survive_meteor, target_count: 1, counters: {kill: 1}}</x:v>
-      </x:c>
-      <x:c r="K4" t="str">
-        <x:v>ItemReward{key: preview_dragon_scale, item: @Item.dragon_scale, count: 1}</x:v>
-      </x:c>
-      <x:c r="L4" t="str">
-        <x:v>start_day: 20, end_day: 90</x:v>
-      </x:c>
-      <x:c r="M4" t="str">
-        <x:v>key: root, text: "The peak is burning.", next: [{key: rally, text: "Gather the raid."} | {key: scout, text: "Find a safer path.", next: [{key: report, text: "Return before dawn."}]}]</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2" t="str">
-        <x:v>Shop ID</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="str">
-        <x:v>Name Text ID</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>Kind</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>Open Day</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
-        <x:v>Close Day</x:v>
-      </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>Stage Gate ID</x:v>
-      </x:c>
-      <x:c r="G1" s="2" t="str">
-        <x:v>Entries</x:v>
-      </x:c>
-      <x:c r="H1" s="2" t="str">
-        <x:v>Currencies</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>shop_starter</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>@Text.shop_starter_name</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>General</x:v>
-      </x:c>
-      <x:c r="D2" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="F2" t="str">
-        <x:v>_</x:v>
-      </x:c>
-      <x:c r="G2" t="str">
-        <x:v>{item: @Item.healing_potion, price: 35, stock: 20, unlock_level: 1, required_quest: _, discount_by_day: {1: 0, 7: 10}} | {item: @Equipment.iron_sword, price: 120, stock: 1, unlock_level: 1, required_quest: @Quest.quest_first_blade, discount_by_day: {1: 0}}</x:v>
-      </x:c>
-      <x:c r="H2" t="str">
-        <x:v>gold</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>shop_arcane</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>@Text.shop_arcane_name</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>Event</x:v>
-      </x:c>
-      <x:c r="D3" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="E3" t="n">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="F3" t="str">
-        <x:v>@Stage.stage_arcane_tower</x:v>
-      </x:c>
-      <x:c r="G3" t="str">
-        <x:v>{item: @Equipment.flame_staff, price: 760, stock: 1, unlock_level: 12, required_quest: @Quest.quest_mage_trial, discount_by_day: {1: 0, 14: 15}} | {item: @Item.phoenix_feather, price: 1800, stock: 5, unlock_level: 18, required_quest: @Quest.quest_mage_trial, discount_by_day: {1: 0}}</x:v>
-      </x:c>
-      <x:c r="H3" t="str">
-        <x:v>gold | event_token</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>shop_raid</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>@Text.shop_raid_name</x:v>
-      </x:c>
-      <x:c r="C4" t="str">
-        <x:v>Raid</x:v>
-      </x:c>
-      <x:c r="D4" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E4" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="F4" t="str">
-        <x:v>@Stage.stage_dragon_peak</x:v>
-      </x:c>
-      <x:c r="G4" t="str">
-        <x:v>{item: @Item.dragon_scale, price: 5200, stock: 4, unlock_level: 45, required_quest: @Quest.quest_dragon_raid, discount_by_day: {1: 0}} | {item: @Equipment.meteor_staff, price: 2600, stock: 1, unlock_level: 45, required_quest: @Quest.quest_dragon_raid, discount_by_day: {1: 0, 30: 20}}</x:v>
-      </x:c>
-      <x:c r="H4" t="str">
-        <x:v>gold | raid_token</x:v>
+      <x:c r="D14" t="str">
+        <x:v>quest title</x:v>
+      </x:c>
+      <x:c r="E14" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>quest | raid</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>shop_starter_name</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>新手补给</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Starter Supply</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>shop name</x:v>
+      </x:c>
+      <x:c r="E15" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>shop | general</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>shop_arcane_name</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>秘法商店</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Arcane Shop</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>shop name</x:v>
+      </x:c>
+      <x:c r="E16" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>shop | event</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>shop_raid_name</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>讨伐补给</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Raid Supply</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>shop name</x:v>
+      </x:c>
+      <x:c r="E17" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>shop | raid</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: document enum placeholders and method builtins
</commit_message>
<xml_diff>
--- a/examples/rpg/data/rpg.xlsx
+++ b/examples/rpg/data/rpg.xlsx
@@ -450,7 +450,7 @@
     <t>Weapon | Armor</t>
   </si>
   <si>
-    <t>shape: cone, params: {range: 2.0, angle: 90.0}</t>
+    <t>shape: cone, parameters: {range: 2.0, angle: 90.0}</t>
   </si>
   <si>
     <t>fireball</t>
@@ -471,7 +471,7 @@
     <t>Weapon | Accessory</t>
   </si>
   <si>
-    <t>shape: circle, params: {range: 8.0, radius: 2.5}</t>
+    <t>shape: circle, parameters: {range: 8.0, radius: 2.5}</t>
   </si>
   <si>
     <t>meteor</t>
@@ -489,7 +489,7 @@
     <t>0 | 50 | 100</t>
   </si>
   <si>
-    <t>shape: circle, params: {range: 12.0, radius: 5.0}</t>
+    <t>shape: circle, parameters: {range: 12.0, radius: 5.0}</t>
   </si>
   <si>
     <t>battle_trance</t>
@@ -504,7 +504,7 @@
     <t>0 | 5 | 10</t>
   </si>
   <si>
-    <t>shape: self, params: {range: 0.0, duration: 12.0}</t>
+    <t>shape: self, parameters: {range: 0.0, duration: 12.0}</t>
   </si>
   <si>
     <t>Monster ID</t>

</xml_diff>